<commit_message>
Build-Skripte für die Excel-Fassung ins Repo aufnehmen
tools/extract_data.js liest die Checklisten aus der Web-App,
tools/build_xlsx.py erzeugt daraus Instandhaltungs-Audit.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5PqJuB3Png3kBCTuPDxEq
</commit_message>
<xml_diff>
--- a/Instandhaltungs-Audit.xlsx
+++ b/Instandhaltungs-Audit.xlsx
@@ -2676,11 +2676,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="87161038"/>
-        <c:axId val="90712029"/>
+        <c:axId val="62229826"/>
+        <c:axId val="35701826"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="87161038"/>
+        <c:axId val="62229826"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2712,7 +2712,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90712029"/>
+        <c:crossAx val="35701826"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2720,7 +2720,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90712029"/>
+        <c:axId val="35701826"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2764,7 +2764,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87161038"/>
+        <c:crossAx val="62229826"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3211,11 +3211,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="83066920"/>
-        <c:axId val="77136142"/>
+        <c:axId val="82825357"/>
+        <c:axId val="12285162"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83066920"/>
+        <c:axId val="82825357"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3247,7 +3247,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77136142"/>
+        <c:crossAx val="12285162"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3255,7 +3255,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77136142"/>
+        <c:axId val="12285162"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3297,7 +3297,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83066920"/>
+        <c:crossAx val="82825357"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3487,11 +3487,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="33556856"/>
-        <c:axId val="30955390"/>
+        <c:axId val="42947941"/>
+        <c:axId val="46634138"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="33556856"/>
+        <c:axId val="42947941"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3523,7 +3523,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30955390"/>
+        <c:crossAx val="46634138"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3531,7 +3531,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30955390"/>
+        <c:axId val="46634138"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3573,7 +3573,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33556856"/>
+        <c:crossAx val="42947941"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3745,11 +3745,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57780026"/>
-        <c:axId val="46528933"/>
+        <c:axId val="6818153"/>
+        <c:axId val="89944710"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57780026"/>
+        <c:axId val="6818153"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3781,7 +3781,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46528933"/>
+        <c:crossAx val="89944710"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3789,7 +3789,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46528933"/>
+        <c:axId val="89944710"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3831,7 +3831,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57780026"/>
+        <c:crossAx val="6818153"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4006,11 +4006,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="91134615"/>
-        <c:axId val="46050456"/>
+        <c:axId val="16890619"/>
+        <c:axId val="17119"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91134615"/>
+        <c:axId val="16890619"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4042,7 +4042,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46050456"/>
+        <c:crossAx val="17119"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4050,7 +4050,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46050456"/>
+        <c:axId val="17119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4084,7 +4084,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91134615"/>
+        <c:crossAx val="16890619"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4244,11 +4244,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="88633042"/>
-        <c:axId val="40460530"/>
+        <c:axId val="74146090"/>
+        <c:axId val="25354673"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88633042"/>
+        <c:axId val="74146090"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4280,7 +4280,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40460530"/>
+        <c:crossAx val="25354673"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4288,7 +4288,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40460530"/>
+        <c:axId val="25354673"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4322,7 +4322,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88633042"/>
+        <c:crossAx val="74146090"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4485,11 +4485,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="76768102"/>
-        <c:axId val="88579655"/>
+        <c:axId val="88856414"/>
+        <c:axId val="85569881"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="76768102"/>
+        <c:axId val="88856414"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4521,7 +4521,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88579655"/>
+        <c:crossAx val="85569881"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4529,7 +4529,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88579655"/>
+        <c:axId val="85569881"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4563,7 +4563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76768102"/>
+        <c:crossAx val="88856414"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4720,11 +4720,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95456558"/>
-        <c:axId val="13521162"/>
+        <c:axId val="36229330"/>
+        <c:axId val="19325637"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95456558"/>
+        <c:axId val="36229330"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -4756,7 +4756,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13521162"/>
+        <c:crossAx val="19325637"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4764,7 +4764,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13521162"/>
+        <c:axId val="19325637"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -4798,7 +4798,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95456558"/>
+        <c:crossAx val="36229330"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7683,16 +7683,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" error="Bitte ein Datum eingeben (TT.MM.JJJJ)." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6 H12:H50" type="date">
-      <formula1>36526</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" error="Bitte N.I.O, bed. OK, OK oder n. b. wählen." errorStyle="stop" errorTitle="Bewertung" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E12:E50" type="list">
       <formula1>"N.I.O,bed. OK,OK,n. b."</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I12:I50" type="list">
       <formula1>"ja,nein"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="Bitte ein Datum eingeben (TT.MM.JJJJ)." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6 H12:H50" type="date">
+      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -8428,16 +8428,16 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
+    <dataValidation allowBlank="true" error="Bitte ein Datum eingeben (TT.MM.JJJJ)." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6 H12:H24" type="date">
+      <formula1>36526</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="true" error="Bitte N.I.O, bed. OK, OK oder n. b. wählen." errorStyle="stop" errorTitle="Bewertung" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E12:E24" type="list">
       <formula1>"N.I.O,bed. OK,OK,n. b."</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I12:I24" type="list">
       <formula1>"ja,nein"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" error="Bitte ein Datum eingeben (TT.MM.JJJJ)." errorStyle="stop" operator="greaterThan" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6 H12:H24" type="date">
-      <formula1>36526</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>